<commit_message>
is to update v001 and v002
</commit_message>
<xml_diff>
--- a/F_grouping/reference/backtesting_score.xlsx
+++ b/F_grouping/reference/backtesting_score.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="138" uniqueCount="133">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="133">
   <si>
     <t>factor_name</t>
   </si>
@@ -52,15 +52,15 @@
     <t>I002</t>
   </si>
   <si>
+    <t>W004_I_signal</t>
+  </si>
+  <si>
     <t>W001</t>
   </si>
   <si>
     <t>W002</t>
   </si>
   <si>
-    <t>W004_I_signal</t>
-  </si>
-  <si>
     <t>G004</t>
   </si>
   <si>
@@ -70,73 +70,73 @@
     <t>I004</t>
   </si>
   <si>
+    <t>W004_P_signal</t>
+  </si>
+  <si>
+    <t>O005</t>
+  </si>
+  <si>
+    <t>P002</t>
+  </si>
+  <si>
+    <t>V002</t>
+  </si>
+  <si>
+    <t>V004</t>
+  </si>
+  <si>
+    <t>I003</t>
+  </si>
+  <si>
+    <t>I024</t>
+  </si>
+  <si>
+    <t>G002</t>
+  </si>
+  <si>
+    <t>L005</t>
+  </si>
+  <si>
+    <t>W003_I</t>
+  </si>
+  <si>
+    <t>W004_I</t>
+  </si>
+  <si>
+    <t>F005</t>
+  </si>
+  <si>
+    <t>P016</t>
+  </si>
+  <si>
+    <t>W004_signal</t>
+  </si>
+  <si>
+    <t>F002</t>
+  </si>
+  <si>
+    <t>W003_W</t>
+  </si>
+  <si>
+    <t>L023</t>
+  </si>
+  <si>
+    <t>L025</t>
+  </si>
+  <si>
+    <t>L011</t>
+  </si>
+  <si>
+    <t>G003</t>
+  </si>
+  <si>
+    <t>V003</t>
+  </si>
+  <si>
+    <t>V016</t>
+  </si>
+  <si>
     <t>P001</t>
-  </si>
-  <si>
-    <t>W004_P_signal</t>
-  </si>
-  <si>
-    <t>O005</t>
-  </si>
-  <si>
-    <t>P002</t>
-  </si>
-  <si>
-    <t>V002</t>
-  </si>
-  <si>
-    <t>V004</t>
-  </si>
-  <si>
-    <t>I003</t>
-  </si>
-  <si>
-    <t>I024</t>
-  </si>
-  <si>
-    <t>G002</t>
-  </si>
-  <si>
-    <t>L005</t>
-  </si>
-  <si>
-    <t>W003_I</t>
-  </si>
-  <si>
-    <t>W004_I</t>
-  </si>
-  <si>
-    <t>F005</t>
-  </si>
-  <si>
-    <t>P016</t>
-  </si>
-  <si>
-    <t>W004_signal</t>
-  </si>
-  <si>
-    <t>F002</t>
-  </si>
-  <si>
-    <t>W003_W</t>
-  </si>
-  <si>
-    <t>L023</t>
-  </si>
-  <si>
-    <t>L025</t>
-  </si>
-  <si>
-    <t>L011</t>
-  </si>
-  <si>
-    <t>G003</t>
-  </si>
-  <si>
-    <t>V003</t>
-  </si>
-  <si>
-    <t>V016</t>
   </si>
   <si>
     <t>V001</t>
@@ -744,7 +744,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I130"/>
+  <dimension ref="A1:I125"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:9">
@@ -865,7 +865,7 @@
     </row>
     <row r="5" spans="1:9">
       <c r="A5" t="s">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B5" t="b">
         <v>1</v>
@@ -889,12 +889,12 @@
         <v>4</v>
       </c>
       <c r="I5">
-        <v>0.525</v>
+        <v>0.521875</v>
       </c>
     </row>
     <row r="6" spans="1:9">
       <c r="A6" t="s">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B6" t="b">
         <v>1</v>
@@ -918,12 +918,12 @@
         <v>4</v>
       </c>
       <c r="I6">
-        <v>0.525</v>
+        <v>0.51875</v>
       </c>
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B7" t="b">
         <v>1</v>
@@ -947,12 +947,12 @@
         <v>4</v>
       </c>
       <c r="I7">
-        <v>0.525</v>
+        <v>0.51875</v>
       </c>
     </row>
     <row r="8" spans="1:9">
       <c r="A8" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B8" t="b">
         <v>1</v>
@@ -976,12 +976,12 @@
         <v>4</v>
       </c>
       <c r="I8">
-        <v>0.521875</v>
+        <v>0.5145833333333332</v>
       </c>
     </row>
     <row r="9" spans="1:9">
       <c r="A9" t="s">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="B9" t="b">
         <v>1</v>
@@ -990,10 +990,10 @@
         <v>1</v>
       </c>
       <c r="D9" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E9" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F9" t="b">
         <v>0</v>
@@ -1005,12 +1005,12 @@
         <v>4</v>
       </c>
       <c r="I9">
-        <v>0.51875</v>
+        <v>0.5104166666666666</v>
       </c>
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="B10" t="b">
         <v>1</v>
@@ -1019,10 +1019,10 @@
         <v>1</v>
       </c>
       <c r="D10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F10" t="b">
         <v>0</v>
@@ -1034,12 +1034,12 @@
         <v>4</v>
       </c>
       <c r="I10">
-        <v>0.51875</v>
+        <v>0.509375</v>
       </c>
     </row>
     <row r="11" spans="1:9">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B11" t="b">
         <v>1</v>
@@ -1063,12 +1063,12 @@
         <v>4</v>
       </c>
       <c r="I11">
-        <v>0.5145833333333332</v>
+        <v>0.5052083333333334</v>
       </c>
     </row>
     <row r="12" spans="1:9">
       <c r="A12" t="s">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="B12" t="b">
         <v>1</v>
@@ -1092,24 +1092,24 @@
         <v>4</v>
       </c>
       <c r="I12">
-        <v>0.5104166666666666</v>
+        <v>0.478125</v>
       </c>
     </row>
     <row r="13" spans="1:9">
       <c r="A13" t="s">
-        <v>17</v>
+        <v>20</v>
       </c>
       <c r="B13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C13" t="b">
         <v>1</v>
       </c>
       <c r="D13" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F13" t="b">
         <v>0</v>
@@ -1118,15 +1118,15 @@
         <v>1</v>
       </c>
       <c r="H13">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I13">
-        <v>0.509375</v>
+        <v>0.5354166666666667</v>
       </c>
     </row>
     <row r="14" spans="1:9">
       <c r="A14" t="s">
-        <v>18</v>
+        <v>21</v>
       </c>
       <c r="B14" t="b">
         <v>1</v>
@@ -1135,7 +1135,7 @@
         <v>1</v>
       </c>
       <c r="D14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" t="b">
         <v>0</v>
@@ -1147,15 +1147,15 @@
         <v>1</v>
       </c>
       <c r="H14">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I14">
-        <v>0.5052083333333334</v>
+        <v>0.5302083333333333</v>
       </c>
     </row>
     <row r="15" spans="1:9">
       <c r="A15" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="B15" t="b">
         <v>1</v>
@@ -1164,7 +1164,7 @@
         <v>1</v>
       </c>
       <c r="D15" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E15" t="b">
         <v>0</v>
@@ -1176,15 +1176,15 @@
         <v>1</v>
       </c>
       <c r="H15">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I15">
-        <v>0.5052083333333334</v>
+        <v>0.5302083333333333</v>
       </c>
     </row>
     <row r="16" spans="1:9">
       <c r="A16" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="B16" t="b">
         <v>1</v>
@@ -1196,7 +1196,7 @@
         <v>0</v>
       </c>
       <c r="E16" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F16" t="b">
         <v>0</v>
@@ -1205,24 +1205,24 @@
         <v>1</v>
       </c>
       <c r="H16">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I16">
-        <v>0.478125</v>
+        <v>0.5291666666666667</v>
       </c>
     </row>
     <row r="17" spans="1:9">
       <c r="A17" t="s">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="B17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C17" t="b">
         <v>1</v>
       </c>
       <c r="D17" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E17" t="b">
         <v>0</v>
@@ -1237,12 +1237,12 @@
         <v>3</v>
       </c>
       <c r="I17">
-        <v>0.5354166666666667</v>
+        <v>0.5291666666666667</v>
       </c>
     </row>
     <row r="18" spans="1:9">
       <c r="A18" t="s">
-        <v>22</v>
+        <v>25</v>
       </c>
       <c r="B18" t="b">
         <v>1</v>
@@ -1266,12 +1266,12 @@
         <v>3</v>
       </c>
       <c r="I18">
-        <v>0.5302083333333333</v>
+        <v>0.5291666666666666</v>
       </c>
     </row>
     <row r="19" spans="1:9">
       <c r="A19" t="s">
-        <v>23</v>
+        <v>26</v>
       </c>
       <c r="B19" t="b">
         <v>1</v>
@@ -1295,12 +1295,12 @@
         <v>3</v>
       </c>
       <c r="I19">
-        <v>0.5302083333333333</v>
+        <v>0.5229166666666666</v>
       </c>
     </row>
     <row r="20" spans="1:9">
       <c r="A20" t="s">
-        <v>24</v>
+        <v>27</v>
       </c>
       <c r="B20" t="b">
         <v>1</v>
@@ -1324,12 +1324,12 @@
         <v>3</v>
       </c>
       <c r="I20">
-        <v>0.5291666666666667</v>
+        <v>0.521875</v>
       </c>
     </row>
     <row r="21" spans="1:9">
       <c r="A21" t="s">
-        <v>25</v>
+        <v>28</v>
       </c>
       <c r="B21" t="b">
         <v>1</v>
@@ -1353,12 +1353,12 @@
         <v>3</v>
       </c>
       <c r="I21">
-        <v>0.5291666666666667</v>
+        <v>0.521875</v>
       </c>
     </row>
     <row r="22" spans="1:9">
       <c r="A22" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="B22" t="b">
         <v>1</v>
@@ -1382,15 +1382,15 @@
         <v>3</v>
       </c>
       <c r="I22">
-        <v>0.5291666666666666</v>
+        <v>0.5166666666666666</v>
       </c>
     </row>
     <row r="23" spans="1:9">
       <c r="A23" t="s">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="B23" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C23" t="b">
         <v>1</v>
@@ -1399,7 +1399,7 @@
         <v>0</v>
       </c>
       <c r="E23" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
@@ -1411,12 +1411,12 @@
         <v>3</v>
       </c>
       <c r="I23">
-        <v>0.528125</v>
+        <v>0.5114583333333333</v>
       </c>
     </row>
     <row r="24" spans="1:9">
       <c r="A24" t="s">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="B24" t="b">
         <v>1</v>
@@ -1440,15 +1440,15 @@
         <v>3</v>
       </c>
       <c r="I24">
-        <v>0.5229166666666666</v>
+        <v>0.5114583333333333</v>
       </c>
     </row>
     <row r="25" spans="1:9">
       <c r="A25" t="s">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="B25" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C25" t="b">
         <v>1</v>
@@ -1457,7 +1457,7 @@
         <v>0</v>
       </c>
       <c r="E25" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F25" t="b">
         <v>0</v>
@@ -1469,12 +1469,12 @@
         <v>3</v>
       </c>
       <c r="I25">
-        <v>0.521875</v>
+        <v>0.5104166666666666</v>
       </c>
     </row>
     <row r="26" spans="1:9">
       <c r="A26" t="s">
-        <v>29</v>
+        <v>33</v>
       </c>
       <c r="B26" t="b">
         <v>1</v>
@@ -1498,12 +1498,12 @@
         <v>3</v>
       </c>
       <c r="I26">
-        <v>0.521875</v>
+        <v>0.509375</v>
       </c>
     </row>
     <row r="27" spans="1:9">
       <c r="A27" t="s">
-        <v>30</v>
+        <v>34</v>
       </c>
       <c r="B27" t="b">
         <v>1</v>
@@ -1527,15 +1527,15 @@
         <v>3</v>
       </c>
       <c r="I27">
-        <v>0.5166666666666666</v>
+        <v>0.5083333333333334</v>
       </c>
     </row>
     <row r="28" spans="1:9">
       <c r="A28" t="s">
-        <v>31</v>
+        <v>35</v>
       </c>
       <c r="B28" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C28" t="b">
         <v>1</v>
@@ -1544,7 +1544,7 @@
         <v>0</v>
       </c>
       <c r="E28" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F28" t="b">
         <v>0</v>
@@ -1556,12 +1556,12 @@
         <v>3</v>
       </c>
       <c r="I28">
-        <v>0.5114583333333333</v>
+        <v>0.5083333333333334</v>
       </c>
     </row>
     <row r="29" spans="1:9">
       <c r="A29" t="s">
-        <v>32</v>
+        <v>36</v>
       </c>
       <c r="B29" t="b">
         <v>1</v>
@@ -1585,15 +1585,15 @@
         <v>3</v>
       </c>
       <c r="I29">
-        <v>0.5114583333333333</v>
+        <v>0.5072916666666666</v>
       </c>
     </row>
     <row r="30" spans="1:9">
       <c r="A30" t="s">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="B30" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C30" t="b">
         <v>1</v>
@@ -1602,7 +1602,7 @@
         <v>0</v>
       </c>
       <c r="E30" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F30" t="b">
         <v>0</v>
@@ -1614,12 +1614,12 @@
         <v>3</v>
       </c>
       <c r="I30">
-        <v>0.5104166666666666</v>
+        <v>0.5062500000000001</v>
       </c>
     </row>
     <row r="31" spans="1:9">
       <c r="A31" t="s">
-        <v>34</v>
+        <v>38</v>
       </c>
       <c r="B31" t="b">
         <v>1</v>
@@ -1643,12 +1643,12 @@
         <v>3</v>
       </c>
       <c r="I31">
-        <v>0.509375</v>
+        <v>0.5062500000000001</v>
       </c>
     </row>
     <row r="32" spans="1:9">
       <c r="A32" t="s">
-        <v>35</v>
+        <v>39</v>
       </c>
       <c r="B32" t="b">
         <v>1</v>
@@ -1672,12 +1672,12 @@
         <v>3</v>
       </c>
       <c r="I32">
-        <v>0.5083333333333334</v>
+        <v>0.5062500000000001</v>
       </c>
     </row>
     <row r="33" spans="1:9">
       <c r="A33" t="s">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="B33" t="b">
         <v>1</v>
@@ -1701,12 +1701,12 @@
         <v>3</v>
       </c>
       <c r="I33">
-        <v>0.5083333333333334</v>
+        <v>0.5052083333333334</v>
       </c>
     </row>
     <row r="34" spans="1:9">
       <c r="A34" t="s">
-        <v>37</v>
+        <v>41</v>
       </c>
       <c r="B34" t="b">
         <v>1</v>
@@ -1730,12 +1730,12 @@
         <v>3</v>
       </c>
       <c r="I34">
-        <v>0.5072916666666666</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="35" spans="1:9">
       <c r="A35" t="s">
-        <v>38</v>
+        <v>42</v>
       </c>
       <c r="B35" t="b">
         <v>1</v>
@@ -1759,12 +1759,12 @@
         <v>3</v>
       </c>
       <c r="I35">
-        <v>0.5062500000000001</v>
+        <v>0.4989583333333334</v>
       </c>
     </row>
     <row r="36" spans="1:9">
       <c r="A36" t="s">
-        <v>39</v>
+        <v>43</v>
       </c>
       <c r="B36" t="b">
         <v>1</v>
@@ -1776,24 +1776,24 @@
         <v>0</v>
       </c>
       <c r="E36" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F36" t="b">
         <v>0</v>
       </c>
       <c r="G36" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H36">
         <v>3</v>
       </c>
       <c r="I36">
-        <v>0.5062500000000001</v>
+        <v>0.4989583333333333</v>
       </c>
     </row>
     <row r="37" spans="1:9">
       <c r="A37" t="s">
-        <v>40</v>
+        <v>44</v>
       </c>
       <c r="B37" t="b">
         <v>1</v>
@@ -1817,12 +1817,12 @@
         <v>3</v>
       </c>
       <c r="I37">
-        <v>0.5062500000000001</v>
+        <v>0.4979166666666666</v>
       </c>
     </row>
     <row r="38" spans="1:9">
       <c r="A38" t="s">
-        <v>18</v>
+        <v>45</v>
       </c>
       <c r="B38" t="b">
         <v>1</v>
@@ -1846,12 +1846,12 @@
         <v>3</v>
       </c>
       <c r="I38">
-        <v>0.5052083333333334</v>
+        <v>0.4958333333333334</v>
       </c>
     </row>
     <row r="39" spans="1:9">
       <c r="A39" t="s">
-        <v>41</v>
+        <v>46</v>
       </c>
       <c r="B39" t="b">
         <v>1</v>
@@ -1863,24 +1863,24 @@
         <v>0</v>
       </c>
       <c r="E39" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F39" t="b">
         <v>0</v>
       </c>
       <c r="G39" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H39">
         <v>3</v>
       </c>
       <c r="I39">
-        <v>0.5</v>
+        <v>0.4947916666666666</v>
       </c>
     </row>
     <row r="40" spans="1:9">
       <c r="A40" t="s">
-        <v>42</v>
+        <v>47</v>
       </c>
       <c r="B40" t="b">
         <v>1</v>
@@ -1904,12 +1904,12 @@
         <v>3</v>
       </c>
       <c r="I40">
-        <v>0.4989583333333334</v>
+        <v>0.4916666666666666</v>
       </c>
     </row>
     <row r="41" spans="1:9">
       <c r="A41" t="s">
-        <v>43</v>
+        <v>48</v>
       </c>
       <c r="B41" t="b">
         <v>1</v>
@@ -1921,24 +1921,24 @@
         <v>0</v>
       </c>
       <c r="E41" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F41" t="b">
         <v>0</v>
       </c>
       <c r="G41" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H41">
         <v>3</v>
       </c>
       <c r="I41">
-        <v>0.4989583333333333</v>
+        <v>0.490625</v>
       </c>
     </row>
     <row r="42" spans="1:9">
       <c r="A42" t="s">
-        <v>44</v>
+        <v>49</v>
       </c>
       <c r="B42" t="b">
         <v>1</v>
@@ -1962,12 +1962,12 @@
         <v>3</v>
       </c>
       <c r="I42">
-        <v>0.4979166666666666</v>
+        <v>0.4885416666666667</v>
       </c>
     </row>
     <row r="43" spans="1:9">
       <c r="A43" t="s">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="B43" t="b">
         <v>1</v>
@@ -1991,12 +1991,12 @@
         <v>3</v>
       </c>
       <c r="I43">
-        <v>0.4958333333333334</v>
+        <v>0.4875</v>
       </c>
     </row>
     <row r="44" spans="1:9">
       <c r="A44" t="s">
-        <v>46</v>
+        <v>51</v>
       </c>
       <c r="B44" t="b">
         <v>1</v>
@@ -2008,24 +2008,24 @@
         <v>0</v>
       </c>
       <c r="E44" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F44" t="b">
         <v>0</v>
       </c>
       <c r="G44" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H44">
         <v>3</v>
       </c>
       <c r="I44">
-        <v>0.4947916666666666</v>
+        <v>0.484375</v>
       </c>
     </row>
     <row r="45" spans="1:9">
       <c r="A45" t="s">
-        <v>47</v>
+        <v>52</v>
       </c>
       <c r="B45" t="b">
         <v>1</v>
@@ -2049,12 +2049,12 @@
         <v>3</v>
       </c>
       <c r="I45">
-        <v>0.4916666666666666</v>
+        <v>0.4802083333333333</v>
       </c>
     </row>
     <row r="46" spans="1:9">
       <c r="A46" t="s">
-        <v>48</v>
+        <v>53</v>
       </c>
       <c r="B46" t="b">
         <v>1</v>
@@ -2078,12 +2078,12 @@
         <v>3</v>
       </c>
       <c r="I46">
-        <v>0.490625</v>
+        <v>0.4770833333333333</v>
       </c>
     </row>
     <row r="47" spans="1:9">
       <c r="A47" t="s">
-        <v>49</v>
+        <v>54</v>
       </c>
       <c r="B47" t="b">
         <v>1</v>
@@ -2101,18 +2101,18 @@
         <v>0</v>
       </c>
       <c r="G47" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H47">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I47">
-        <v>0.4885416666666667</v>
+        <v>0.5291666666666666</v>
       </c>
     </row>
     <row r="48" spans="1:9">
       <c r="A48" t="s">
-        <v>50</v>
+        <v>55</v>
       </c>
       <c r="B48" t="b">
         <v>1</v>
@@ -2130,18 +2130,18 @@
         <v>0</v>
       </c>
       <c r="G48" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H48">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I48">
-        <v>0.4875</v>
+        <v>0.5270833333333332</v>
       </c>
     </row>
     <row r="49" spans="1:9">
       <c r="A49" t="s">
-        <v>51</v>
+        <v>56</v>
       </c>
       <c r="B49" t="b">
         <v>1</v>
@@ -2159,18 +2159,18 @@
         <v>0</v>
       </c>
       <c r="G49" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H49">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I49">
-        <v>0.484375</v>
+        <v>0.5260416666666667</v>
       </c>
     </row>
     <row r="50" spans="1:9">
       <c r="A50" t="s">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="B50" t="b">
         <v>1</v>
@@ -2188,18 +2188,18 @@
         <v>0</v>
       </c>
       <c r="G50" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H50">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I50">
-        <v>0.4802083333333333</v>
+        <v>0.5260416666666667</v>
       </c>
     </row>
     <row r="51" spans="1:9">
       <c r="A51" t="s">
-        <v>53</v>
+        <v>58</v>
       </c>
       <c r="B51" t="b">
         <v>1</v>
@@ -2217,18 +2217,18 @@
         <v>0</v>
       </c>
       <c r="G51" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H51">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="I51">
-        <v>0.4770833333333333</v>
+        <v>0.5239583333333334</v>
       </c>
     </row>
     <row r="52" spans="1:9">
       <c r="A52" t="s">
-        <v>54</v>
+        <v>59</v>
       </c>
       <c r="B52" t="b">
         <v>1</v>
@@ -2252,12 +2252,12 @@
         <v>2</v>
       </c>
       <c r="I52">
-        <v>0.5291666666666666</v>
+        <v>0.5177083333333334</v>
       </c>
     </row>
     <row r="53" spans="1:9">
       <c r="A53" t="s">
-        <v>55</v>
+        <v>60</v>
       </c>
       <c r="B53" t="b">
         <v>1</v>
@@ -2281,12 +2281,12 @@
         <v>2</v>
       </c>
       <c r="I53">
-        <v>0.5270833333333332</v>
+        <v>0.5166666666666667</v>
       </c>
     </row>
     <row r="54" spans="1:9">
       <c r="A54" t="s">
-        <v>56</v>
+        <v>61</v>
       </c>
       <c r="B54" t="b">
         <v>1</v>
@@ -2310,12 +2310,12 @@
         <v>2</v>
       </c>
       <c r="I54">
-        <v>0.5260416666666667</v>
+        <v>0.515625</v>
       </c>
     </row>
     <row r="55" spans="1:9">
       <c r="A55" t="s">
-        <v>57</v>
+        <v>62</v>
       </c>
       <c r="B55" t="b">
         <v>1</v>
@@ -2339,12 +2339,12 @@
         <v>2</v>
       </c>
       <c r="I55">
-        <v>0.5260416666666667</v>
+        <v>0.5135416666666666</v>
       </c>
     </row>
     <row r="56" spans="1:9">
       <c r="A56" t="s">
-        <v>58</v>
+        <v>63</v>
       </c>
       <c r="B56" t="b">
         <v>1</v>
@@ -2368,12 +2368,12 @@
         <v>2</v>
       </c>
       <c r="I56">
-        <v>0.5239583333333334</v>
+        <v>0.5135416666666666</v>
       </c>
     </row>
     <row r="57" spans="1:9">
       <c r="A57" t="s">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="B57" t="b">
         <v>1</v>
@@ -2397,12 +2397,12 @@
         <v>2</v>
       </c>
       <c r="I57">
-        <v>0.5177083333333334</v>
+        <v>0.5104166666666667</v>
       </c>
     </row>
     <row r="58" spans="1:9">
       <c r="A58" t="s">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="B58" t="b">
         <v>1</v>
@@ -2426,12 +2426,12 @@
         <v>2</v>
       </c>
       <c r="I58">
-        <v>0.5166666666666667</v>
+        <v>0.5083333333333333</v>
       </c>
     </row>
     <row r="59" spans="1:9">
       <c r="A59" t="s">
-        <v>61</v>
+        <v>66</v>
       </c>
       <c r="B59" t="b">
         <v>1</v>
@@ -2455,12 +2455,12 @@
         <v>2</v>
       </c>
       <c r="I59">
-        <v>0.515625</v>
+        <v>0.5083333333333333</v>
       </c>
     </row>
     <row r="60" spans="1:9">
       <c r="A60" t="s">
-        <v>62</v>
+        <v>67</v>
       </c>
       <c r="B60" t="b">
         <v>1</v>
@@ -2484,12 +2484,12 @@
         <v>2</v>
       </c>
       <c r="I60">
-        <v>0.5135416666666666</v>
+        <v>0.5062500000000001</v>
       </c>
     </row>
     <row r="61" spans="1:9">
       <c r="A61" t="s">
-        <v>63</v>
+        <v>68</v>
       </c>
       <c r="B61" t="b">
         <v>1</v>
@@ -2513,12 +2513,12 @@
         <v>2</v>
       </c>
       <c r="I61">
-        <v>0.5135416666666666</v>
+        <v>0.50625</v>
       </c>
     </row>
     <row r="62" spans="1:9">
       <c r="A62" t="s">
-        <v>64</v>
+        <v>69</v>
       </c>
       <c r="B62" t="b">
         <v>1</v>
@@ -2542,12 +2542,12 @@
         <v>2</v>
       </c>
       <c r="I62">
-        <v>0.5104166666666667</v>
+        <v>0.503125</v>
       </c>
     </row>
     <row r="63" spans="1:9">
       <c r="A63" t="s">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="B63" t="b">
         <v>1</v>
@@ -2571,12 +2571,12 @@
         <v>2</v>
       </c>
       <c r="I63">
-        <v>0.5083333333333333</v>
+        <v>0.503125</v>
       </c>
     </row>
     <row r="64" spans="1:9">
       <c r="A64" t="s">
-        <v>66</v>
+        <v>71</v>
       </c>
       <c r="B64" t="b">
         <v>1</v>
@@ -2600,12 +2600,12 @@
         <v>2</v>
       </c>
       <c r="I64">
-        <v>0.5083333333333333</v>
+        <v>0.503125</v>
       </c>
     </row>
     <row r="65" spans="1:9">
       <c r="A65" t="s">
-        <v>67</v>
+        <v>72</v>
       </c>
       <c r="B65" t="b">
         <v>1</v>
@@ -2629,12 +2629,12 @@
         <v>2</v>
       </c>
       <c r="I65">
-        <v>0.5062500000000001</v>
+        <v>0.5020833333333333</v>
       </c>
     </row>
     <row r="66" spans="1:9">
       <c r="A66" t="s">
-        <v>68</v>
+        <v>73</v>
       </c>
       <c r="B66" t="b">
         <v>1</v>
@@ -2658,12 +2658,12 @@
         <v>2</v>
       </c>
       <c r="I66">
-        <v>0.50625</v>
+        <v>0.5010416666666667</v>
       </c>
     </row>
     <row r="67" spans="1:9">
       <c r="A67" t="s">
-        <v>69</v>
+        <v>74</v>
       </c>
       <c r="B67" t="b">
         <v>1</v>
@@ -2687,12 +2687,12 @@
         <v>2</v>
       </c>
       <c r="I67">
-        <v>0.503125</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="68" spans="1:9">
       <c r="A68" t="s">
-        <v>70</v>
+        <v>75</v>
       </c>
       <c r="B68" t="b">
         <v>1</v>
@@ -2716,12 +2716,12 @@
         <v>2</v>
       </c>
       <c r="I68">
-        <v>0.503125</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="69" spans="1:9">
       <c r="A69" t="s">
-        <v>71</v>
+        <v>76</v>
       </c>
       <c r="B69" t="b">
         <v>1</v>
@@ -2745,12 +2745,12 @@
         <v>2</v>
       </c>
       <c r="I69">
-        <v>0.503125</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="70" spans="1:9">
       <c r="A70" t="s">
-        <v>72</v>
+        <v>77</v>
       </c>
       <c r="B70" t="b">
         <v>1</v>
@@ -2774,12 +2774,12 @@
         <v>2</v>
       </c>
       <c r="I70">
-        <v>0.5020833333333333</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="71" spans="1:9">
       <c r="A71" t="s">
-        <v>73</v>
+        <v>78</v>
       </c>
       <c r="B71" t="b">
         <v>1</v>
@@ -2803,12 +2803,12 @@
         <v>2</v>
       </c>
       <c r="I71">
-        <v>0.5010416666666667</v>
+        <v>0.4989583333333333</v>
       </c>
     </row>
     <row r="72" spans="1:9">
       <c r="A72" t="s">
-        <v>74</v>
+        <v>79</v>
       </c>
       <c r="B72" t="b">
         <v>1</v>
@@ -2832,12 +2832,12 @@
         <v>2</v>
       </c>
       <c r="I72">
-        <v>0.5</v>
+        <v>0.496875</v>
       </c>
     </row>
     <row r="73" spans="1:9">
       <c r="A73" t="s">
-        <v>75</v>
+        <v>80</v>
       </c>
       <c r="B73" t="b">
         <v>1</v>
@@ -2861,12 +2861,12 @@
         <v>2</v>
       </c>
       <c r="I73">
-        <v>0.5</v>
+        <v>0.4958333333333334</v>
       </c>
     </row>
     <row r="74" spans="1:9">
       <c r="A74" t="s">
-        <v>76</v>
+        <v>81</v>
       </c>
       <c r="B74" t="b">
         <v>1</v>
@@ -2890,12 +2890,12 @@
         <v>2</v>
       </c>
       <c r="I74">
-        <v>0.5</v>
+        <v>0.4958333333333334</v>
       </c>
     </row>
     <row r="75" spans="1:9">
       <c r="A75" t="s">
-        <v>77</v>
+        <v>82</v>
       </c>
       <c r="B75" t="b">
         <v>1</v>
@@ -2919,12 +2919,12 @@
         <v>2</v>
       </c>
       <c r="I75">
-        <v>0.5</v>
+        <v>0.4958333333333334</v>
       </c>
     </row>
     <row r="76" spans="1:9">
       <c r="A76" t="s">
-        <v>78</v>
+        <v>83</v>
       </c>
       <c r="B76" t="b">
         <v>1</v>
@@ -2948,12 +2948,12 @@
         <v>2</v>
       </c>
       <c r="I76">
-        <v>0.4989583333333333</v>
+        <v>0.4958333333333333</v>
       </c>
     </row>
     <row r="77" spans="1:9">
       <c r="A77" t="s">
-        <v>79</v>
+        <v>84</v>
       </c>
       <c r="B77" t="b">
         <v>1</v>
@@ -2977,12 +2977,12 @@
         <v>2</v>
       </c>
       <c r="I77">
-        <v>0.496875</v>
+        <v>0.4947916666666667</v>
       </c>
     </row>
     <row r="78" spans="1:9">
       <c r="A78" t="s">
-        <v>80</v>
+        <v>85</v>
       </c>
       <c r="B78" t="b">
         <v>1</v>
@@ -3006,12 +3006,12 @@
         <v>2</v>
       </c>
       <c r="I78">
-        <v>0.4958333333333334</v>
+        <v>0.4947916666666667</v>
       </c>
     </row>
     <row r="79" spans="1:9">
       <c r="A79" t="s">
-        <v>81</v>
+        <v>86</v>
       </c>
       <c r="B79" t="b">
         <v>1</v>
@@ -3035,12 +3035,12 @@
         <v>2</v>
       </c>
       <c r="I79">
-        <v>0.4958333333333334</v>
+        <v>0.4947916666666667</v>
       </c>
     </row>
     <row r="80" spans="1:9">
       <c r="A80" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="B80" t="b">
         <v>1</v>
@@ -3064,12 +3064,12 @@
         <v>2</v>
       </c>
       <c r="I80">
-        <v>0.4958333333333334</v>
+        <v>0.4947916666666667</v>
       </c>
     </row>
     <row r="81" spans="1:9">
       <c r="A81" t="s">
-        <v>83</v>
+        <v>88</v>
       </c>
       <c r="B81" t="b">
         <v>1</v>
@@ -3093,12 +3093,12 @@
         <v>2</v>
       </c>
       <c r="I81">
-        <v>0.4958333333333333</v>
+        <v>0.4927083333333334</v>
       </c>
     </row>
     <row r="82" spans="1:9">
       <c r="A82" t="s">
-        <v>84</v>
+        <v>89</v>
       </c>
       <c r="B82" t="b">
         <v>1</v>
@@ -3122,12 +3122,12 @@
         <v>2</v>
       </c>
       <c r="I82">
-        <v>0.4947916666666667</v>
+        <v>0.4927083333333333</v>
       </c>
     </row>
     <row r="83" spans="1:9">
       <c r="A83" t="s">
-        <v>85</v>
+        <v>90</v>
       </c>
       <c r="B83" t="b">
         <v>1</v>
@@ -3151,12 +3151,12 @@
         <v>2</v>
       </c>
       <c r="I83">
-        <v>0.4947916666666667</v>
+        <v>0.4927083333333333</v>
       </c>
     </row>
     <row r="84" spans="1:9">
       <c r="A84" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="B84" t="b">
         <v>1</v>
@@ -3180,12 +3180,12 @@
         <v>2</v>
       </c>
       <c r="I84">
-        <v>0.4947916666666667</v>
+        <v>0.4927083333333333</v>
       </c>
     </row>
     <row r="85" spans="1:9">
       <c r="A85" t="s">
-        <v>87</v>
+        <v>92</v>
       </c>
       <c r="B85" t="b">
         <v>1</v>
@@ -3209,12 +3209,12 @@
         <v>2</v>
       </c>
       <c r="I85">
-        <v>0.4947916666666667</v>
+        <v>0.4916666666666667</v>
       </c>
     </row>
     <row r="86" spans="1:9">
       <c r="A86" t="s">
-        <v>88</v>
+        <v>93</v>
       </c>
       <c r="B86" t="b">
         <v>1</v>
@@ -3238,12 +3238,12 @@
         <v>2</v>
       </c>
       <c r="I86">
-        <v>0.4927083333333334</v>
+        <v>0.4916666666666666</v>
       </c>
     </row>
     <row r="87" spans="1:9">
       <c r="A87" t="s">
-        <v>89</v>
+        <v>94</v>
       </c>
       <c r="B87" t="b">
         <v>1</v>
@@ -3267,15 +3267,15 @@
         <v>2</v>
       </c>
       <c r="I87">
-        <v>0.4927083333333333</v>
+        <v>0.4895833333333333</v>
       </c>
     </row>
     <row r="88" spans="1:9">
       <c r="A88" t="s">
-        <v>90</v>
+        <v>95</v>
       </c>
       <c r="B88" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C88" t="b">
         <v>1</v>
@@ -3290,18 +3290,18 @@
         <v>0</v>
       </c>
       <c r="G88" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="H88">
         <v>2</v>
       </c>
       <c r="I88">
-        <v>0.4927083333333333</v>
+        <v>0.4885416666666666</v>
       </c>
     </row>
     <row r="89" spans="1:9">
       <c r="A89" t="s">
-        <v>91</v>
+        <v>96</v>
       </c>
       <c r="B89" t="b">
         <v>1</v>
@@ -3325,12 +3325,12 @@
         <v>2</v>
       </c>
       <c r="I89">
-        <v>0.4927083333333333</v>
+        <v>0.4885416666666666</v>
       </c>
     </row>
     <row r="90" spans="1:9">
       <c r="A90" t="s">
-        <v>92</v>
+        <v>97</v>
       </c>
       <c r="B90" t="b">
         <v>1</v>
@@ -3354,12 +3354,12 @@
         <v>2</v>
       </c>
       <c r="I90">
-        <v>0.4916666666666667</v>
+        <v>0.4864583333333333</v>
       </c>
     </row>
     <row r="91" spans="1:9">
       <c r="A91" t="s">
-        <v>93</v>
+        <v>98</v>
       </c>
       <c r="B91" t="b">
         <v>1</v>
@@ -3383,12 +3383,12 @@
         <v>2</v>
       </c>
       <c r="I91">
-        <v>0.4916666666666666</v>
+        <v>0.4854166666666666</v>
       </c>
     </row>
     <row r="92" spans="1:9">
       <c r="A92" t="s">
-        <v>94</v>
+        <v>99</v>
       </c>
       <c r="B92" t="b">
         <v>1</v>
@@ -3412,15 +3412,15 @@
         <v>2</v>
       </c>
       <c r="I92">
-        <v>0.4895833333333333</v>
+        <v>0.484375</v>
       </c>
     </row>
     <row r="93" spans="1:9">
       <c r="A93" t="s">
-        <v>95</v>
+        <v>100</v>
       </c>
       <c r="B93" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C93" t="b">
         <v>1</v>
@@ -3435,18 +3435,18 @@
         <v>0</v>
       </c>
       <c r="G93" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="H93">
         <v>2</v>
       </c>
       <c r="I93">
-        <v>0.4885416666666666</v>
+        <v>0.484375</v>
       </c>
     </row>
     <row r="94" spans="1:9">
       <c r="A94" t="s">
-        <v>96</v>
+        <v>101</v>
       </c>
       <c r="B94" t="b">
         <v>1</v>
@@ -3470,12 +3470,12 @@
         <v>2</v>
       </c>
       <c r="I94">
-        <v>0.4885416666666666</v>
+        <v>0.4833333333333334</v>
       </c>
     </row>
     <row r="95" spans="1:9">
       <c r="A95" t="s">
-        <v>97</v>
+        <v>102</v>
       </c>
       <c r="B95" t="b">
         <v>1</v>
@@ -3499,12 +3499,12 @@
         <v>2</v>
       </c>
       <c r="I95">
-        <v>0.4864583333333333</v>
+        <v>0.4833333333333333</v>
       </c>
     </row>
     <row r="96" spans="1:9">
       <c r="A96" t="s">
-        <v>98</v>
+        <v>103</v>
       </c>
       <c r="B96" t="b">
         <v>1</v>
@@ -3528,12 +3528,12 @@
         <v>2</v>
       </c>
       <c r="I96">
-        <v>0.4854166666666666</v>
+        <v>0.4833333333333333</v>
       </c>
     </row>
     <row r="97" spans="1:9">
       <c r="A97" t="s">
-        <v>99</v>
+        <v>104</v>
       </c>
       <c r="B97" t="b">
         <v>1</v>
@@ -3557,12 +3557,12 @@
         <v>2</v>
       </c>
       <c r="I97">
-        <v>0.484375</v>
+        <v>0.4802083333333334</v>
       </c>
     </row>
     <row r="98" spans="1:9">
       <c r="A98" t="s">
-        <v>100</v>
+        <v>105</v>
       </c>
       <c r="B98" t="b">
         <v>1</v>
@@ -3586,12 +3586,12 @@
         <v>2</v>
       </c>
       <c r="I98">
-        <v>0.484375</v>
+        <v>0.4791666666666667</v>
       </c>
     </row>
     <row r="99" spans="1:9">
       <c r="A99" t="s">
-        <v>101</v>
+        <v>106</v>
       </c>
       <c r="B99" t="b">
         <v>1</v>
@@ -3615,12 +3615,12 @@
         <v>2</v>
       </c>
       <c r="I99">
-        <v>0.4833333333333334</v>
+        <v>0.4770833333333333</v>
       </c>
     </row>
     <row r="100" spans="1:9">
       <c r="A100" t="s">
-        <v>102</v>
+        <v>107</v>
       </c>
       <c r="B100" t="b">
         <v>1</v>
@@ -3644,12 +3644,12 @@
         <v>2</v>
       </c>
       <c r="I100">
-        <v>0.4833333333333333</v>
+        <v>0.4739583333333333</v>
       </c>
     </row>
     <row r="101" spans="1:9">
       <c r="A101" t="s">
-        <v>103</v>
+        <v>108</v>
       </c>
       <c r="B101" t="b">
         <v>1</v>
@@ -3673,18 +3673,18 @@
         <v>2</v>
       </c>
       <c r="I101">
-        <v>0.4833333333333333</v>
+        <v>0.4739583333333333</v>
       </c>
     </row>
     <row r="102" spans="1:9">
       <c r="A102" t="s">
-        <v>104</v>
+        <v>109</v>
       </c>
       <c r="B102" t="b">
         <v>1</v>
       </c>
       <c r="C102" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D102" t="b">
         <v>0</v>
@@ -3699,18 +3699,18 @@
         <v>0</v>
       </c>
       <c r="H102">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I102">
-        <v>0.4802083333333334</v>
+        <v>0.5354166666666667</v>
       </c>
     </row>
     <row r="103" spans="1:9">
       <c r="A103" t="s">
-        <v>105</v>
+        <v>110</v>
       </c>
       <c r="B103" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C103" t="b">
         <v>1</v>
@@ -3728,18 +3728,18 @@
         <v>0</v>
       </c>
       <c r="H103">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I103">
-        <v>0.4791666666666667</v>
+        <v>0.53125</v>
       </c>
     </row>
     <row r="104" spans="1:9">
       <c r="A104" t="s">
-        <v>106</v>
+        <v>111</v>
       </c>
       <c r="B104" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C104" t="b">
         <v>1</v>
@@ -3757,18 +3757,18 @@
         <v>0</v>
       </c>
       <c r="H104">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I104">
-        <v>0.4770833333333333</v>
+        <v>0.5125</v>
       </c>
     </row>
     <row r="105" spans="1:9">
       <c r="A105" t="s">
-        <v>107</v>
+        <v>112</v>
       </c>
       <c r="B105" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C105" t="b">
         <v>1</v>
@@ -3786,18 +3786,18 @@
         <v>0</v>
       </c>
       <c r="H105">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I105">
-        <v>0.4739583333333333</v>
+        <v>0.5104166666666666</v>
       </c>
     </row>
     <row r="106" spans="1:9">
       <c r="A106" t="s">
-        <v>108</v>
+        <v>113</v>
       </c>
       <c r="B106" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C106" t="b">
         <v>1</v>
@@ -3815,21 +3815,21 @@
         <v>0</v>
       </c>
       <c r="H106">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="I106">
-        <v>0.4739583333333333</v>
+        <v>0.5104166666666666</v>
       </c>
     </row>
     <row r="107" spans="1:9">
       <c r="A107" t="s">
-        <v>109</v>
+        <v>114</v>
       </c>
       <c r="B107" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C107" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D107" t="b">
         <v>0</v>
@@ -3847,12 +3847,12 @@
         <v>1</v>
       </c>
       <c r="I107">
-        <v>0.5354166666666667</v>
+        <v>0.5104166666666666</v>
       </c>
     </row>
     <row r="108" spans="1:9">
       <c r="A108" t="s">
-        <v>110</v>
+        <v>115</v>
       </c>
       <c r="B108" t="b">
         <v>0</v>
@@ -3876,12 +3876,12 @@
         <v>1</v>
       </c>
       <c r="I108">
-        <v>0.53125</v>
+        <v>0.5104166666666666</v>
       </c>
     </row>
     <row r="109" spans="1:9">
       <c r="A109" t="s">
-        <v>111</v>
+        <v>116</v>
       </c>
       <c r="B109" t="b">
         <v>0</v>
@@ -3905,12 +3905,12 @@
         <v>1</v>
       </c>
       <c r="I109">
-        <v>0.5125</v>
+        <v>0.5052083333333334</v>
       </c>
     </row>
     <row r="110" spans="1:9">
       <c r="A110" t="s">
-        <v>112</v>
+        <v>117</v>
       </c>
       <c r="B110" t="b">
         <v>0</v>
@@ -3934,18 +3934,18 @@
         <v>1</v>
       </c>
       <c r="I110">
-        <v>0.5104166666666666</v>
+        <v>0.5052083333333334</v>
       </c>
     </row>
     <row r="111" spans="1:9">
       <c r="A111" t="s">
-        <v>113</v>
+        <v>118</v>
       </c>
       <c r="B111" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C111" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D111" t="b">
         <v>0</v>
@@ -3963,18 +3963,18 @@
         <v>1</v>
       </c>
       <c r="I111">
-        <v>0.5104166666666666</v>
+        <v>0.5041666666666667</v>
       </c>
     </row>
     <row r="112" spans="1:9">
       <c r="A112" t="s">
-        <v>114</v>
+        <v>119</v>
       </c>
       <c r="B112" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C112" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D112" t="b">
         <v>0</v>
@@ -3992,18 +3992,18 @@
         <v>1</v>
       </c>
       <c r="I112">
-        <v>0.5104166666666666</v>
+        <v>0.5041666666666667</v>
       </c>
     </row>
     <row r="113" spans="1:9">
       <c r="A113" t="s">
-        <v>115</v>
+        <v>120</v>
       </c>
       <c r="B113" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C113" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D113" t="b">
         <v>0</v>
@@ -4021,18 +4021,18 @@
         <v>1</v>
       </c>
       <c r="I113">
-        <v>0.5104166666666666</v>
+        <v>0.4947916666666667</v>
       </c>
     </row>
     <row r="114" spans="1:9">
       <c r="A114" t="s">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="B114" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C114" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D114" t="b">
         <v>0</v>
@@ -4050,12 +4050,12 @@
         <v>1</v>
       </c>
       <c r="I114">
-        <v>0.5052083333333334</v>
+        <v>0.4927083333333333</v>
       </c>
     </row>
     <row r="115" spans="1:9">
       <c r="A115" t="s">
-        <v>117</v>
+        <v>122</v>
       </c>
       <c r="B115" t="b">
         <v>0</v>
@@ -4079,12 +4079,12 @@
         <v>1</v>
       </c>
       <c r="I115">
-        <v>0.5052083333333334</v>
+        <v>0.4895833333333333</v>
       </c>
     </row>
     <row r="116" spans="1:9">
       <c r="A116" t="s">
-        <v>118</v>
+        <v>123</v>
       </c>
       <c r="B116" t="b">
         <v>1</v>
@@ -4108,18 +4108,18 @@
         <v>1</v>
       </c>
       <c r="I116">
-        <v>0.5041666666666667</v>
+        <v>0.4875</v>
       </c>
     </row>
     <row r="117" spans="1:9">
       <c r="A117" t="s">
-        <v>119</v>
+        <v>124</v>
       </c>
       <c r="B117" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C117" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D117" t="b">
         <v>0</v>
@@ -4137,18 +4137,18 @@
         <v>1</v>
       </c>
       <c r="I117">
-        <v>0.5041666666666667</v>
+        <v>0.4864583333333333</v>
       </c>
     </row>
     <row r="118" spans="1:9">
       <c r="A118" t="s">
-        <v>120</v>
+        <v>125</v>
       </c>
       <c r="B118" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C118" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D118" t="b">
         <v>0</v>
@@ -4166,18 +4166,18 @@
         <v>1</v>
       </c>
       <c r="I118">
-        <v>0.4947916666666667</v>
+        <v>0.4864583333333333</v>
       </c>
     </row>
     <row r="119" spans="1:9">
       <c r="A119" t="s">
-        <v>121</v>
+        <v>126</v>
       </c>
       <c r="B119" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C119" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D119" t="b">
         <v>0</v>
@@ -4195,18 +4195,18 @@
         <v>1</v>
       </c>
       <c r="I119">
-        <v>0.4927083333333333</v>
+        <v>0.4864583333333333</v>
       </c>
     </row>
     <row r="120" spans="1:9">
       <c r="A120" t="s">
-        <v>122</v>
+        <v>127</v>
       </c>
       <c r="B120" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C120" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D120" t="b">
         <v>0</v>
@@ -4224,12 +4224,12 @@
         <v>1</v>
       </c>
       <c r="I120">
-        <v>0.4895833333333333</v>
+        <v>0.4854166666666666</v>
       </c>
     </row>
     <row r="121" spans="1:9">
       <c r="A121" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="B121" t="b">
         <v>1</v>
@@ -4253,18 +4253,18 @@
         <v>1</v>
       </c>
       <c r="I121">
-        <v>0.4875</v>
+        <v>0.4760416666666667</v>
       </c>
     </row>
     <row r="122" spans="1:9">
       <c r="A122" t="s">
-        <v>124</v>
+        <v>129</v>
       </c>
       <c r="B122" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C122" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D122" t="b">
         <v>0</v>
@@ -4282,18 +4282,18 @@
         <v>1</v>
       </c>
       <c r="I122">
-        <v>0.4864583333333333</v>
+        <v>0.4614583333333333</v>
       </c>
     </row>
     <row r="123" spans="1:9">
       <c r="A123" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="B123" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C123" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D123" t="b">
         <v>0</v>
@@ -4311,18 +4311,18 @@
         <v>1</v>
       </c>
       <c r="I123">
-        <v>0.4864583333333333</v>
+        <v>0.45</v>
       </c>
     </row>
     <row r="124" spans="1:9">
       <c r="A124" t="s">
-        <v>126</v>
+        <v>131</v>
       </c>
       <c r="B124" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="C124" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="D124" t="b">
         <v>0</v>
@@ -4340,15 +4340,15 @@
         <v>1</v>
       </c>
       <c r="I124">
-        <v>0.4864583333333333</v>
+        <v>0.4260416666666667</v>
       </c>
     </row>
     <row r="125" spans="1:9">
       <c r="A125" t="s">
-        <v>127</v>
+        <v>132</v>
       </c>
       <c r="B125" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C125" t="b">
         <v>0</v>
@@ -4366,154 +4366,9 @@
         <v>0</v>
       </c>
       <c r="H125">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="I125">
-        <v>0.4854166666666666</v>
-      </c>
-    </row>
-    <row r="126" spans="1:9">
-      <c r="A126" t="s">
-        <v>128</v>
-      </c>
-      <c r="B126" t="b">
-        <v>1</v>
-      </c>
-      <c r="C126" t="b">
-        <v>0</v>
-      </c>
-      <c r="D126" t="b">
-        <v>0</v>
-      </c>
-      <c r="E126" t="b">
-        <v>0</v>
-      </c>
-      <c r="F126" t="b">
-        <v>0</v>
-      </c>
-      <c r="G126" t="b">
-        <v>0</v>
-      </c>
-      <c r="H126">
-        <v>1</v>
-      </c>
-      <c r="I126">
-        <v>0.4760416666666667</v>
-      </c>
-    </row>
-    <row r="127" spans="1:9">
-      <c r="A127" t="s">
-        <v>129</v>
-      </c>
-      <c r="B127" t="b">
-        <v>1</v>
-      </c>
-      <c r="C127" t="b">
-        <v>0</v>
-      </c>
-      <c r="D127" t="b">
-        <v>0</v>
-      </c>
-      <c r="E127" t="b">
-        <v>0</v>
-      </c>
-      <c r="F127" t="b">
-        <v>0</v>
-      </c>
-      <c r="G127" t="b">
-        <v>0</v>
-      </c>
-      <c r="H127">
-        <v>1</v>
-      </c>
-      <c r="I127">
-        <v>0.4614583333333333</v>
-      </c>
-    </row>
-    <row r="128" spans="1:9">
-      <c r="A128" t="s">
-        <v>130</v>
-      </c>
-      <c r="B128" t="b">
-        <v>1</v>
-      </c>
-      <c r="C128" t="b">
-        <v>0</v>
-      </c>
-      <c r="D128" t="b">
-        <v>0</v>
-      </c>
-      <c r="E128" t="b">
-        <v>0</v>
-      </c>
-      <c r="F128" t="b">
-        <v>0</v>
-      </c>
-      <c r="G128" t="b">
-        <v>0</v>
-      </c>
-      <c r="H128">
-        <v>1</v>
-      </c>
-      <c r="I128">
-        <v>0.45</v>
-      </c>
-    </row>
-    <row r="129" spans="1:9">
-      <c r="A129" t="s">
-        <v>131</v>
-      </c>
-      <c r="B129" t="b">
-        <v>1</v>
-      </c>
-      <c r="C129" t="b">
-        <v>0</v>
-      </c>
-      <c r="D129" t="b">
-        <v>0</v>
-      </c>
-      <c r="E129" t="b">
-        <v>0</v>
-      </c>
-      <c r="F129" t="b">
-        <v>0</v>
-      </c>
-      <c r="G129" t="b">
-        <v>0</v>
-      </c>
-      <c r="H129">
-        <v>1</v>
-      </c>
-      <c r="I129">
-        <v>0.4260416666666667</v>
-      </c>
-    </row>
-    <row r="130" spans="1:9">
-      <c r="A130" t="s">
-        <v>132</v>
-      </c>
-      <c r="B130" t="b">
-        <v>0</v>
-      </c>
-      <c r="C130" t="b">
-        <v>0</v>
-      </c>
-      <c r="D130" t="b">
-        <v>0</v>
-      </c>
-      <c r="E130" t="b">
-        <v>0</v>
-      </c>
-      <c r="F130" t="b">
-        <v>0</v>
-      </c>
-      <c r="G130" t="b">
-        <v>0</v>
-      </c>
-      <c r="H130">
-        <v>0</v>
-      </c>
-      <c r="I130">
         <v>0.478125</v>
       </c>
     </row>

</xml_diff>